<commit_message>
Mise a jour du 11-08-2026 15:55:17,11
</commit_message>
<xml_diff>
--- a/contenu/Premiere.xlsx
+++ b/contenu/Premiere.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E99CFA1-F302-4CF2-AE4C-593DAA0C7B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D29942-5374-4FAA-833B-2D7F34ADA9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -93,9 +93,6 @@
     <t>Muche</t>
   </si>
   <si>
-    <t>gFKvZoN3H1c</t>
-  </si>
-  <si>
     <t>Niveau 4 YT</t>
   </si>
   <si>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>Niveau 5 DG</t>
+  </si>
+  <si>
+    <t>O_S7nyIq0N8</t>
   </si>
 </sst>
 </file>
@@ -467,16 +467,16 @@
         <v>8</v>
       </c>
       <c r="L1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" t="s">
         <v>18</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>19</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>20</v>
-      </c>
-      <c r="O1" t="s">
-        <v>21</v>
       </c>
       <c r="P1" t="s">
         <v>9</v>
@@ -500,7 +500,7 @@
         <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="J2" t="s">
         <v>12</v>
@@ -524,7 +524,7 @@
         <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Mise a jour du 11-08-2026 22:05:50,77
</commit_message>
<xml_diff>
--- a/contenu/Premiere.xlsx
+++ b/contenu/Premiere.xlsx
@@ -1,37 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D29942-5374-4FAA-833B-2D7F34ADA9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CFB929-40A3-4FA1-B786-9615011F426A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
     <sheet name="Plannification" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -40,7 +26,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+  <si>
+    <t>Préfixe</t>
+  </si>
   <si>
     <t>n° Chapitre</t>
   </si>
@@ -48,7 +37,10 @@
     <t>n° SF</t>
   </si>
   <si>
-    <t>Préfixe</t>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Titre</t>
   </si>
   <si>
     <t>Niveau 1 YT</t>
@@ -57,25 +49,64 @@
     <t>Niveau 1 DG</t>
   </si>
   <si>
+    <t>Niveau 1 fin</t>
+  </si>
+  <si>
     <t>Niveau 2 YT</t>
   </si>
   <si>
     <t>Niveau 2 DG</t>
   </si>
   <si>
+    <t>Niveau 2 fin</t>
+  </si>
+  <si>
     <t>Niveau 3 YT</t>
   </si>
   <si>
     <t>Niveau 3 DG</t>
   </si>
   <si>
+    <t>Niveau 3 fin</t>
+  </si>
+  <si>
+    <t>Niveau 4 YT</t>
+  </si>
+  <si>
+    <t>Niveau 4 DG</t>
+  </si>
+  <si>
+    <t>Niveau 4 fin</t>
+  </si>
+  <si>
+    <t>Niveau 5 YT</t>
+  </si>
+  <si>
+    <t>Niveau 5 DG</t>
+  </si>
+  <si>
+    <t>Niveau 5 fin</t>
+  </si>
+  <si>
     <t>Commentaire</t>
   </si>
   <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Titre</t>
+    <t>T</t>
+  </si>
+  <si>
+    <t>T.SF1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiplier par 1 </t>
+  </si>
+  <si>
+    <t>qrV9v5vRsz4</t>
+  </si>
+  <si>
+    <t>T.SF1.2</t>
+  </si>
+  <si>
+    <t>Diviser par 0</t>
   </si>
   <si>
     <t>AA9_JHSruJ0</t>
@@ -85,27 +116,6 @@
   </si>
   <si>
     <t>x</t>
-  </si>
-  <si>
-    <t>Truc</t>
-  </si>
-  <si>
-    <t>Muche</t>
-  </si>
-  <si>
-    <t>Niveau 4 YT</t>
-  </si>
-  <si>
-    <t>Niveau 4 DG</t>
-  </si>
-  <si>
-    <t>Niveau 5 YT</t>
-  </si>
-  <si>
-    <t>Niveau 5 DG</t>
-  </si>
-  <si>
-    <t>O_S7nyIq0N8</t>
   </si>
 </sst>
 </file>
@@ -143,7 +153,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -425,66 +435,81 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="4" max="4" width="9.765625" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="4" max="4" width="9.765625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="M1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="N1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="O1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="P1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A2">
-        <v>1</v>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>21</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -492,23 +517,22 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="str">
-        <f>A2 &amp; "." &amp;"SF"&amp;B2&amp; "." &amp;C2</f>
-        <v>1.SF1.1</v>
+      <c r="D2" t="s">
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
         <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A3">
-        <v>1</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -516,76 +540,22 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" t="str">
-        <f t="shared" ref="D3:D7" si="0">A3 &amp; "." &amp;"SF"&amp;B3&amp; "." &amp;C3</f>
-        <v>1.SF1.2</v>
+      <c r="D3" t="s">
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4" t="str">
-        <f t="shared" si="0"/>
-        <v>1.SF1.3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="str">
-        <f t="shared" si="0"/>
-        <v>1.SF2.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6" t="str">
-        <f t="shared" si="0"/>
-        <v>1.SF2.2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="B7">
-        <v>3</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7" t="str">
-        <f t="shared" si="0"/>
-        <v>1.SF3.1</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="H3">
+        <v>3153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="D4"/>
+      <c r="E4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -593,21 +563,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE5B9D5-5188-414E-BDD4-28B2C3DFC193}">
-  <dimension ref="A1:G7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" style="1"/>
+    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.15234375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.07421875" style="1"/>
+    <col min="3" max="3" width="11.07421875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.07421875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>28</v>
       </c>
       <c r="C1" s="2">
         <v>46244</v>
@@ -626,79 +597,42 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="str">
-        <f>Liste!D2</f>
-        <v>1.SF1.1</v>
-      </c>
-      <c r="B2" s="1" t="str">
-        <f>Liste!E2</f>
-        <v>Truc</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>14</v>
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2"/>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="str">
-        <f>Liste!D3</f>
-        <v>1.SF1.2</v>
-      </c>
-      <c r="B3" s="1" t="str">
-        <f>Liste!E3</f>
-        <v>Muche</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>14</v>
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="str">
-        <f>Liste!D4</f>
-        <v>1.SF1.3</v>
-      </c>
-      <c r="B4" s="1">
-        <f>Liste!E4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="str">
-        <f>Liste!D5</f>
-        <v>1.SF2.1</v>
-      </c>
-      <c r="B5" s="1">
-        <f>Liste!E5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="str">
-        <f>Liste!D6</f>
-        <v>1.SF2.2</v>
-      </c>
-      <c r="B6" s="1">
-        <f>Liste!E6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="str">
-        <f>Liste!D7</f>
-        <v>1.SF3.1</v>
-      </c>
-      <c r="B7" s="1">
-        <f>Liste!E7</f>
-        <v>0</v>
-      </c>
+      <c r="A4"/>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="F4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>